<commit_message>
ran analysis on outputs
</commit_message>
<xml_diff>
--- a/outputs/batch/loan_batch_2025-04-11_14-27-40/batch_analysis/combined_results.xlsx
+++ b/outputs/batch/loan_batch_2025-04-11_14-27-40/batch_analysis/combined_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ac15ec0ad8aeca88/Documents/Desktop/Master_Thesis/MasterThesisCode/outputs/batch/loan_batch_2025-04-11_14-27-40/batch_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_D1B55B6EFC93996906754F48B4DED98C0601DB6A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_D1B55B6EFC93996906754F244C5CEAA00601DB6A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B6030EE-57F7-483B-8FB9-13FFAE46A066}"/>
   <bookViews>
-    <workbookView xWindow="32040" yWindow="-10530" windowWidth="21600" windowHeight="11295" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="33060" yWindow="-4605" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="combined_results" sheetId="1" r:id="rId1"/>
@@ -60219,8 +60219,8 @@
   <dimension ref="A1:L61"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="6" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>

</xml_diff>